<commit_message>
Demande EGYDE gardée en Excel : onglet lié à Saisie dans Fiches_clients.xlsx
Remplace le modèle Word EGYDE. Les colonnes EGYDE de « Fiches clients » sont retirées.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4uAx6hF6wT34v3AuaM46U
</commit_message>
<xml_diff>
--- a/Fiches_clients.xlsx
+++ b/Fiches_clients.xlsx
@@ -8,11 +8,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saisie" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiches clients" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demande EGYDE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
   </externalReferences>
   <definedNames>
     <definedName name="Choix1">'[1]Fiche rens. client Air Med '!$A$3</definedName>
@@ -27,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,8 +91,30 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="9"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color theme="1"/>
+      <sz val="9"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -113,8 +136,20 @@
         <fgColor rgb="FFFFF9E0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1900A8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -137,6 +172,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -145,7 +195,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -163,6 +213,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -242,6 +317,93 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>0</col>
+      <colOff>142875</colOff>
+      <row>0</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>3</col>
+      <colOff>161290</colOff>
+      <row>0</row>
+      <rowOff>781050</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 1" descr="logo messer.gif"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="140970" y="49530"/>
+          <a:ext cx="2154555" cy="727710"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>5</col>
+      <colOff>1400175</colOff>
+      <row>0</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>6</col>
+      <colOff>618490</colOff>
+      <row>0</row>
+      <rowOff>885797</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 2" descr="Logo 2Gi-Technologie_RVB.png"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="5617845" y="49530"/>
+          <a:ext cx="849630" cy="838807"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
@@ -1447,7 +1609,7 @@
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>DEMANDE EGYDE – SITE  (modèle Demande EGYDE uniquement ; client, adresse, CP et ville = INFOS CLIENT)</t>
+          <t>DEMANDE EGYDE – SITE  (onglet Demande EGYDE ; client, adresse, CP et ville = INFOS CLIENT)</t>
         </is>
       </c>
     </row>
@@ -1909,49 +2071,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BT2"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="12" min="1" max="33"/>
-    <col width="18" customWidth="1" style="12" min="34" max="34"/>
-    <col width="18" customWidth="1" style="12" min="35" max="35"/>
-    <col width="18" customWidth="1" style="12" min="36" max="36"/>
-    <col width="18" customWidth="1" style="12" min="37" max="37"/>
-    <col width="18" customWidth="1" style="12" min="38" max="38"/>
-    <col width="18" customWidth="1" style="12" min="39" max="39"/>
-    <col width="18" customWidth="1" style="12" min="40" max="40"/>
-    <col width="18" customWidth="1" style="12" min="41" max="41"/>
-    <col width="18" customWidth="1" style="12" min="42" max="42"/>
-    <col width="18" customWidth="1" style="12" min="43" max="43"/>
-    <col width="18" customWidth="1" style="12" min="44" max="44"/>
-    <col width="18" customWidth="1" style="12" min="45" max="45"/>
-    <col width="18" customWidth="1" style="12" min="46" max="46"/>
-    <col width="18" customWidth="1" style="12" min="47" max="47"/>
-    <col width="18" customWidth="1" style="12" min="48" max="48"/>
-    <col width="18" customWidth="1" style="12" min="49" max="49"/>
-    <col width="18" customWidth="1" style="12" min="50" max="50"/>
-    <col width="18" customWidth="1" style="12" min="51" max="51"/>
-    <col width="18" customWidth="1" style="12" min="52" max="52"/>
-    <col width="18" customWidth="1" style="12" min="53" max="53"/>
-    <col width="18" customWidth="1" style="12" min="54" max="54"/>
-    <col width="18" customWidth="1" style="12" min="55" max="55"/>
-    <col width="18" customWidth="1" style="12" min="56" max="56"/>
-    <col width="18" customWidth="1" style="12" min="57" max="57"/>
-    <col width="18" customWidth="1" style="12" min="58" max="58"/>
-    <col width="18" customWidth="1" style="12" min="59" max="59"/>
-    <col width="18" customWidth="1" style="12" min="60" max="60"/>
-    <col width="18" customWidth="1" style="12" min="61" max="61"/>
-    <col width="18" customWidth="1" style="12" min="62" max="62"/>
-    <col width="18" customWidth="1" style="12" min="63" max="63"/>
-    <col width="18" customWidth="1" style="12" min="64" max="64"/>
-    <col width="18" customWidth="1" style="12" min="65" max="65"/>
-    <col width="18" customWidth="1" style="12" min="66" max="66"/>
-    <col width="18" customWidth="1" style="12" min="67" max="67"/>
-    <col width="18" customWidth="1" style="12" min="68" max="68"/>
-    <col width="18" customWidth="1" style="12" min="69" max="69"/>
-    <col width="18" customWidth="1" style="12" min="70" max="70"/>
-    <col width="18" customWidth="1" style="12" min="71" max="71"/>
-    <col width="18" customWidth="1" style="12" min="72" max="72"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2120,201 +2243,6 @@
           <t>P_FLUIDEX</t>
         </is>
       </c>
-      <c r="AH1" s="5" t="inlineStr">
-        <is>
-          <t>E_DateDemande</t>
-        </is>
-      </c>
-      <c r="AI1" s="5" t="inlineStr">
-        <is>
-          <t>E_DateMES</t>
-        </is>
-      </c>
-      <c r="AJ1" s="5" t="inlineStr">
-        <is>
-          <t>E_NomSite</t>
-        </is>
-      </c>
-      <c r="AK1" s="5" t="inlineStr">
-        <is>
-          <t>E_TypeSite</t>
-        </is>
-      </c>
-      <c r="AL1" s="5" t="inlineStr">
-        <is>
-          <t>E_TelSite</t>
-        </is>
-      </c>
-      <c r="AM1" s="5" t="inlineStr">
-        <is>
-          <t>E_NumIdentification</t>
-        </is>
-      </c>
-      <c r="AN1" s="5" t="inlineStr">
-        <is>
-          <t>E_NumEsclave</t>
-        </is>
-      </c>
-      <c r="AO1" s="5" t="inlineStr">
-        <is>
-          <t>E_Astreinte</t>
-        </is>
-      </c>
-      <c r="AP1" s="5" t="inlineStr">
-        <is>
-          <t>E_SourcePrincipale</t>
-        </is>
-      </c>
-      <c r="AQ1" s="5" t="inlineStr">
-        <is>
-          <t>E_SourceAttente</t>
-        </is>
-      </c>
-      <c r="AR1" s="5" t="inlineStr">
-        <is>
-          <t>E_SourceSecours</t>
-        </is>
-      </c>
-      <c r="AS1" s="5" t="inlineStr">
-        <is>
-          <t>E_Commercial</t>
-        </is>
-      </c>
-      <c r="AT1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_Nom</t>
-        </is>
-      </c>
-      <c r="AU1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_Prenom</t>
-        </is>
-      </c>
-      <c r="AV1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_Mail</t>
-        </is>
-      </c>
-      <c r="AW1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_Tel</t>
-        </is>
-      </c>
-      <c r="AX1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_Service</t>
-        </is>
-      </c>
-      <c r="AY1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_Identifiant</t>
-        </is>
-      </c>
-      <c r="AZ1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_MotDePasse</t>
-        </is>
-      </c>
-      <c r="BA1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_TypeAcces</t>
-        </is>
-      </c>
-      <c r="BB1" s="5" t="inlineStr">
-        <is>
-          <t>E_C1_AjoutAlarme</t>
-        </is>
-      </c>
-      <c r="BC1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_Nom</t>
-        </is>
-      </c>
-      <c r="BD1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_Prenom</t>
-        </is>
-      </c>
-      <c r="BE1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_Mail</t>
-        </is>
-      </c>
-      <c r="BF1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_Tel</t>
-        </is>
-      </c>
-      <c r="BG1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_Service</t>
-        </is>
-      </c>
-      <c r="BH1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_Identifiant</t>
-        </is>
-      </c>
-      <c r="BI1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_MotDePasse</t>
-        </is>
-      </c>
-      <c r="BJ1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_TypeAcces</t>
-        </is>
-      </c>
-      <c r="BK1" s="5" t="inlineStr">
-        <is>
-          <t>E_C2_AjoutAlarme</t>
-        </is>
-      </c>
-      <c r="BL1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_Nom</t>
-        </is>
-      </c>
-      <c r="BM1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_Prenom</t>
-        </is>
-      </c>
-      <c r="BN1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_Mail</t>
-        </is>
-      </c>
-      <c r="BO1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_Tel</t>
-        </is>
-      </c>
-      <c r="BP1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_Service</t>
-        </is>
-      </c>
-      <c r="BQ1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_Identifiant</t>
-        </is>
-      </c>
-      <c r="BR1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_MotDePasse</t>
-        </is>
-      </c>
-      <c r="BS1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_TypeAcces</t>
-        </is>
-      </c>
-      <c r="BT1" s="5" t="inlineStr">
-        <is>
-          <t>E_C3_AjoutAlarme</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -2447,162 +2375,6 @@
       </c>
       <c r="AG2">
         <f>IF(Saisie!$B$39="","","X")</f>
-        <v/>
-      </c>
-      <c r="AH2">
-        <f>IF(Saisie!$B$42="","",TEXT(DAY(Saisie!$B$42),"00")&amp;"/"&amp;TEXT(MONTH(Saisie!$B$42),"00")&amp;"/"&amp;YEAR(Saisie!$B$42))</f>
-        <v/>
-      </c>
-      <c r="AI2">
-        <f>IF(Saisie!$B$43="","",TEXT(DAY(Saisie!$B$43),"00")&amp;"/"&amp;TEXT(MONTH(Saisie!$B$43),"00")&amp;"/"&amp;YEAR(Saisie!$B$43))</f>
-        <v/>
-      </c>
-      <c r="AJ2">
-        <f>Saisie!$B$44&amp;""</f>
-        <v/>
-      </c>
-      <c r="AK2">
-        <f>Saisie!$B$45&amp;""</f>
-        <v/>
-      </c>
-      <c r="AL2">
-        <f>Saisie!$B$46&amp;""</f>
-        <v/>
-      </c>
-      <c r="AM2">
-        <f>Saisie!$B$47&amp;""</f>
-        <v/>
-      </c>
-      <c r="AN2">
-        <f>Saisie!$B$48&amp;""</f>
-        <v/>
-      </c>
-      <c r="AO2">
-        <f>Saisie!$B$49&amp;""</f>
-        <v/>
-      </c>
-      <c r="AP2">
-        <f>Saisie!$B$50&amp;""</f>
-        <v/>
-      </c>
-      <c r="AQ2">
-        <f>Saisie!$B$51&amp;""</f>
-        <v/>
-      </c>
-      <c r="AR2">
-        <f>Saisie!$B$52&amp;""</f>
-        <v/>
-      </c>
-      <c r="AS2">
-        <f>Saisie!$B$53&amp;""</f>
-        <v/>
-      </c>
-      <c r="AT2">
-        <f>Saisie!$B$56&amp;""</f>
-        <v/>
-      </c>
-      <c r="AU2">
-        <f>Saisie!$B$57&amp;""</f>
-        <v/>
-      </c>
-      <c r="AV2">
-        <f>Saisie!$B$58&amp;""</f>
-        <v/>
-      </c>
-      <c r="AW2">
-        <f>Saisie!$B$59&amp;""</f>
-        <v/>
-      </c>
-      <c r="AX2">
-        <f>Saisie!$B$60&amp;""</f>
-        <v/>
-      </c>
-      <c r="AY2">
-        <f>Saisie!$B$61&amp;""</f>
-        <v/>
-      </c>
-      <c r="AZ2">
-        <f>Saisie!$B$62&amp;""</f>
-        <v/>
-      </c>
-      <c r="BA2">
-        <f>Saisie!$B$63&amp;""</f>
-        <v/>
-      </c>
-      <c r="BB2">
-        <f>Saisie!$B$64&amp;""</f>
-        <v/>
-      </c>
-      <c r="BC2">
-        <f>Saisie!$B$67&amp;""</f>
-        <v/>
-      </c>
-      <c r="BD2">
-        <f>Saisie!$B$68&amp;""</f>
-        <v/>
-      </c>
-      <c r="BE2">
-        <f>Saisie!$B$69&amp;""</f>
-        <v/>
-      </c>
-      <c r="BF2">
-        <f>Saisie!$B$70&amp;""</f>
-        <v/>
-      </c>
-      <c r="BG2">
-        <f>Saisie!$B$71&amp;""</f>
-        <v/>
-      </c>
-      <c r="BH2">
-        <f>Saisie!$B$72&amp;""</f>
-        <v/>
-      </c>
-      <c r="BI2">
-        <f>Saisie!$B$73&amp;""</f>
-        <v/>
-      </c>
-      <c r="BJ2">
-        <f>Saisie!$B$74&amp;""</f>
-        <v/>
-      </c>
-      <c r="BK2">
-        <f>Saisie!$B$75&amp;""</f>
-        <v/>
-      </c>
-      <c r="BL2">
-        <f>Saisie!$B$78&amp;""</f>
-        <v/>
-      </c>
-      <c r="BM2">
-        <f>Saisie!$B$79&amp;""</f>
-        <v/>
-      </c>
-      <c r="BN2">
-        <f>Saisie!$B$80&amp;""</f>
-        <v/>
-      </c>
-      <c r="BO2">
-        <f>Saisie!$B$81&amp;""</f>
-        <v/>
-      </c>
-      <c r="BP2">
-        <f>Saisie!$B$82&amp;""</f>
-        <v/>
-      </c>
-      <c r="BQ2">
-        <f>Saisie!$B$83&amp;""</f>
-        <v/>
-      </c>
-      <c r="BR2">
-        <f>Saisie!$B$84&amp;""</f>
-        <v/>
-      </c>
-      <c r="BS2">
-        <f>Saisie!$B$85&amp;""</f>
-        <v/>
-      </c>
-      <c r="BT2">
-        <f>Saisie!$B$86&amp;""</f>
         <v/>
       </c>
     </row>
@@ -2612,6 +2384,599 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21.453125" customWidth="1" style="12" min="1" max="1"/>
+    <col width="7.6328125" customWidth="1" style="12" min="2" max="2"/>
+    <col width="1.90625" customWidth="1" style="12" min="3" max="3"/>
+    <col width="10.6328125" customWidth="1" style="12" min="4" max="4"/>
+    <col width="19.90625" customWidth="1" style="12" min="5" max="5"/>
+    <col width="23.6328125" customWidth="1" style="12" min="6" max="6"/>
+    <col width="14.08984375" customWidth="1" style="12" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="72.75" customHeight="1" s="12"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Nom du Site client :</t>
+        </is>
+      </c>
+      <c r="B2" s="14">
+        <f>IF(Saisie!$B$4="","",Saisie!$B$4)</f>
+        <v/>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Date de la demande :</t>
+        </is>
+      </c>
+      <c r="G2" s="15">
+        <f>IF(Saisie!$B$42="","",Saisie!$B$42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Adresse</t>
+        </is>
+      </c>
+      <c r="B3" s="16">
+        <f>IF(Saisie!$B$5="","",Saisie!$B$5)</f>
+        <v/>
+      </c>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Date de M.E.S. souhaitée :</t>
+        </is>
+      </c>
+      <c r="G3" s="15">
+        <f>IF(Saisie!$B$43="","",Saisie!$B$43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="12" customHeight="1" s="12">
+      <c r="B4" s="17" t="n"/>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>(3 jours ouvrés minimum si type existant)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>cp</t>
+        </is>
+      </c>
+      <c r="B5" s="16">
+        <f>IF(Saisie!$B$6="","",Saisie!$B$6)</f>
+        <v/>
+      </c>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="18" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ville</t>
+        </is>
+      </c>
+      <c r="B6" s="20">
+        <f>IF(Saisie!$B$7="","",Saisie!$B$7)</f>
+        <v/>
+      </c>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="16" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Création (à remplir seulement pour la demande d'intégation d'un nouveau Site)</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="21" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Nom du Site :</t>
+        </is>
+      </c>
+      <c r="B8" s="22">
+        <f>IF(Saisie!$B$44="","",Saisie!$B$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Type de Site :</t>
+        </is>
+      </c>
+      <c r="B9" s="14">
+        <f>IF(Saisie!$B$45="","",Saisie!$B$45)</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SOURCE PRINCIPALE </t>
+        </is>
+      </c>
+      <c r="G9" s="16">
+        <f>IF(Saisie!$B$50="","",Saisie!$B$50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>N° De Téléphone :</t>
+        </is>
+      </c>
+      <c r="B10" s="14">
+        <f>IF(Saisie!$B$46="","",Saisie!$B$46)</f>
+        <v/>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SOURCE ATTENTE</t>
+        </is>
+      </c>
+      <c r="G10" s="16">
+        <f>IF(Saisie!$B$51="","",Saisie!$B$51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>N° Identification :</t>
+        </is>
+      </c>
+      <c r="B11" s="22">
+        <f>IF(Saisie!$B$47="","",Saisie!$B$47)</f>
+        <v/>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SOURCE SECOURS</t>
+        </is>
+      </c>
+      <c r="G11" s="16">
+        <f>IF(Saisie!$B$52="","",Saisie!$B$52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N° Esclave : </t>
+        </is>
+      </c>
+      <c r="B12" s="23">
+        <f>IF(Saisie!$B$48="","",Saisie!$B$48)</f>
+        <v/>
+      </c>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="23" t="n"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Commercial responsable</t>
+        </is>
+      </c>
+      <c r="G12" s="16">
+        <f>IF(Saisie!$B$53="","",Saisie!$B$53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>N° ASTREINTE</t>
+        </is>
+      </c>
+      <c r="B13" s="14">
+        <f>IF(Saisie!$B$49="","",Saisie!$B$49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Contact Client (à remplir à la création ou pour ajout nouvel utilisateur)</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="21" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Nom :</t>
+        </is>
+      </c>
+      <c r="B16" s="14">
+        <f>IF(Saisie!$B$56="","",Saisie!$B$56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Prénom :</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>IF(Saisie!$B$57="","",Saisie!$B$57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Adresse Mail :</t>
+        </is>
+      </c>
+      <c r="B18" s="25">
+        <f>IF(Saisie!$B$58="","",Saisie!$B$58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>N° De Téléphone :</t>
+        </is>
+      </c>
+      <c r="B19" s="14">
+        <f>IF(Saisie!$B$59="","",Saisie!$B$59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Service : </t>
+        </is>
+      </c>
+      <c r="B20" s="14">
+        <f>IF(Saisie!$B$60="","",Saisie!$B$60)</f>
+        <v/>
+      </c>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="14" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Identifiant :</t>
+        </is>
+      </c>
+      <c r="B21" s="22">
+        <f>IF(Saisie!$B$61="","",Saisie!$B$61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mot de Passe :</t>
+        </is>
+      </c>
+      <c r="B22" s="22">
+        <f>IF(Saisie!$B$62="","",Saisie!$B$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Type d'accès Client :</t>
+        </is>
+      </c>
+      <c r="B23" s="22">
+        <f>IF(Saisie!$B$63="","",Saisie!$B$63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ajout alarme</t>
+        </is>
+      </c>
+      <c r="B24" s="22">
+        <f>IF(Saisie!$B$64="","",Saisie!$B$64)</f>
+        <v/>
+      </c>
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="22" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="22" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Nom :</t>
+        </is>
+      </c>
+      <c r="B26" s="14">
+        <f>IF(Saisie!$B$67="","",Saisie!$B$67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="12">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Prénom :</t>
+        </is>
+      </c>
+      <c r="B27" s="14">
+        <f>IF(Saisie!$B$68="","",Saisie!$B$68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Adresse Mail :</t>
+        </is>
+      </c>
+      <c r="B28" s="25">
+        <f>IF(Saisie!$B$69="","",Saisie!$B$69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>N° De Téléphone :</t>
+        </is>
+      </c>
+      <c r="B29" s="14">
+        <f>IF(Saisie!$B$70="","",Saisie!$B$70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Service : </t>
+        </is>
+      </c>
+      <c r="B30" s="14">
+        <f>IF(Saisie!$B$71="","",Saisie!$B$71)</f>
+        <v/>
+      </c>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Identifiant :</t>
+        </is>
+      </c>
+      <c r="B31" s="26">
+        <f>IF(Saisie!$B$72="","",Saisie!$B$72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Mot de Passe :</t>
+        </is>
+      </c>
+      <c r="B32" s="22">
+        <f>IF(Saisie!$B$73="","",Saisie!$B$73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Type d'accès Client :</t>
+        </is>
+      </c>
+      <c r="B33" s="22">
+        <f>IF(Saisie!$B$74="","",Saisie!$B$74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ajout alarme</t>
+        </is>
+      </c>
+      <c r="B34" s="22">
+        <f>IF(Saisie!$B$75="","",Saisie!$B$75)</f>
+        <v/>
+      </c>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="22" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="22" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Nom :</t>
+        </is>
+      </c>
+      <c r="B36" s="14">
+        <f>IF(Saisie!$B$78="","",Saisie!$B$78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Prénom :</t>
+        </is>
+      </c>
+      <c r="B37" s="14">
+        <f>IF(Saisie!$B$79="","",Saisie!$B$79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Adresse Mail :</t>
+        </is>
+      </c>
+      <c r="B38" s="25">
+        <f>IF(Saisie!$B$80="","",Saisie!$B$80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>N° De Téléphone :</t>
+        </is>
+      </c>
+      <c r="B39" s="14">
+        <f>IF(Saisie!$B$81="","",Saisie!$B$81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Service : </t>
+        </is>
+      </c>
+      <c r="B40" s="14">
+        <f>IF(Saisie!$B$82="","",Saisie!$B$82)</f>
+        <v/>
+      </c>
+      <c r="C40" s="14" t="n"/>
+      <c r="D40" s="14" t="n"/>
+      <c r="E40" s="14" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Identifiant :</t>
+        </is>
+      </c>
+      <c r="B41" s="22">
+        <f>IF(Saisie!$B$83="","",Saisie!$B$83)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Mot de Passe :</t>
+        </is>
+      </c>
+      <c r="B42" s="22">
+        <f>IF(Saisie!$B$84="","",Saisie!$B$84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Type d'accès Client :</t>
+        </is>
+      </c>
+      <c r="B43" s="22">
+        <f>IF(Saisie!$B$85="","",Saisie!$B$85)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ajout alarme</t>
+        </is>
+      </c>
+      <c r="B44" s="22">
+        <f>IF(Saisie!$B$86="","",Saisie!$B$86)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="30">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B28:E28"/>
+  </mergeCells>
+  <pageMargins left="0.41" right="0.4" top="0.58" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2675,7 +3040,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>6. Section « DEMANDE EGYDE » (en bas de Saisie) : ne sert qu’au modèle Demande EGYDE. Le nom du site client, l’adresse, le CP et la ville sont repris des INFOS CLIENT.</t>
+          <t>6. Demande EGYDE : remplis la section « DEMANDE EGYDE » en bas de Saisie, l’onglet « Demande EGYDE » se remplit tout seul (nom du site client, adresse, CP et ville repris des INFOS CLIENT). Imprime ou envoie cet onglet.</t>
         </is>
       </c>
     </row>

</xml_diff>